<commit_message>
Build source-backed financial review dashboard
</commit_message>
<xml_diff>
--- a/data/raw/capital_markets_monthly.xlsx
+++ b/data/raw/capital_markets_monthly.xlsx
@@ -19,8 +19,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Underwriting Revenue'!$A$1:$P$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trading Revenue'!$A$1:$P$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Structuring Fee'!$A$1:$P$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Syndication Fee'!$A$1:$P$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Operating Expense'!$A$1:$P$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Syndication Fee'!$A$1:$P$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Operating Expense'!$A$1:$P$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -458,7 +458,7 @@
   <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -479,12 +479,12 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Scenario</t>
+          <t>Plan Scenario</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Apr-25</t>
+          <t>Apr_25</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
@@ -619,9 +619,6 @@
       <c r="B3" t="n">
         <v>2.213</v>
       </c>
-      <c r="C3" t="n">
-        <v>2.219</v>
-      </c>
       <c r="D3" t="n">
         <v>2.09</v>
       </c>
@@ -717,7 +714,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Prior Year</t>
+          <t xml:space="preserve"> prior year </t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -781,7 +778,7 @@
   <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -802,12 +799,12 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Scenario</t>
+          <t>Plan Scenario</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Apr-25</t>
+          <t>Apr_25</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
@@ -1060,9 +1057,6 @@
       </c>
       <c r="G5" t="n">
         <v>2.188</v>
-      </c>
-      <c r="H5" t="n">
-        <v>2.316</v>
       </c>
       <c r="I5" t="n">
         <v>2.474</v>
@@ -1104,7 +1098,7 @@
   <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -1125,12 +1119,12 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Scenario</t>
+          <t>Plan Scenario</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Apr-25</t>
+          <t>Apr_25</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
@@ -1226,7 +1220,7 @@
         <v>1.701</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>1.751</v>
+        <v>35.02</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>1.871</v>
@@ -1427,7 +1421,7 @@
   <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -1448,12 +1442,12 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Scenario</t>
+          <t>Plan Scenario</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Apr-25</t>
+          <t>Apr_25</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
@@ -1634,7 +1628,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Forecast</t>
+          <t xml:space="preserve"> forecast </t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -1747,10 +1741,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -1771,12 +1765,12 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Scenario</t>
+          <t>Plan Scenario</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Apr-25</t>
+          <t>Apr_25</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
@@ -2058,8 +2052,60 @@
         <v>0.535</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>0.639</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.638</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>0.598</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0.555</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0.5590000000000001</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0.634</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>0.596</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>0.5610000000000001</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>0.549</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>0.5669999999999999</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>0.737</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P5"/>
+  <autoFilter ref="A1:P6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2070,10 +2116,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -2094,12 +2140,12 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Scenario</t>
+          <t>Plan Scenario</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Apr-25</t>
+          <t>Apr_25</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
@@ -2308,7 +2354,7 @@
         <v>3.556</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>3.612</v>
+        <v>57.792</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>3.536</v>
@@ -2381,8 +2427,60 @@
         <v>3.677</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>3.624</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>3.414</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>3.206</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>3.175</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>3.403</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>3.592</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>3.665</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>3.585</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>3.223</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>3.155</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>3.202</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>3.968</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P5"/>
+  <autoFilter ref="A1:P6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>